<commit_message>
rerun everything from empty output folders; results unchanged
</commit_message>
<xml_diff>
--- a/01_Processing/Figures/S01_QC/c_data/s01_qc.xlsx
+++ b/01_Processing/Figures/S01_QC/c_data/s01_qc.xlsx
@@ -152,7 +152,7 @@
     <t>arm</t>
   </si>
   <si>
-    <t>Study group of the participant (HR or LR), or the cluster that replaces it in a cluster arc.</t>
+    <t>Study group of the participant (HR or LR), or the cluster that replaces it in a cluster grouping.</t>
   </si>
   <si>
     <t>timepoint</t>
@@ -12014,28 +12014,28 @@
     <t>filter</t>
   </si>
   <si>
-    <t>01_Trunk/01_Protein_Filtering/c_data/protein_filtering.xlsx</t>
-  </si>
-  <si>
-    <t>36e4851076be5936c6ea1094c0e9b8a0</t>
+    <t>01_Processing/01_Protein_Filtering/c_data/protein_filtering.xlsx</t>
+  </si>
+  <si>
+    <t>4854fa7ac6d2b74a44ea62851a66ea96</t>
   </si>
   <si>
     <t>normalize</t>
   </si>
   <si>
-    <t>01_Trunk/02_Normalisation/c_data/normalisation.xlsx</t>
-  </si>
-  <si>
-    <t>661b5b8fd32af563512193b5db7c04c3</t>
+    <t>01_Processing/02_Normalisation/c_data/normalisation.xlsx</t>
+  </si>
+  <si>
+    <t>3f7dcfb017ee1077ac79f1a11c4cab5f</t>
   </si>
   <si>
     <t>quantify</t>
   </si>
   <si>
-    <t>01_Trunk/03_Quantification/c_data/quantification.xlsx</t>
-  </si>
-  <si>
-    <t>9e6ea46d26a72e4ac1120f2fdf0afb0e</t>
+    <t>01_Processing/03_Quantification/c_data/quantification.xlsx</t>
+  </si>
+  <si>
+    <t>cdd28d73ea380e8e956c212adbcd2d74</t>
   </si>
   <si>
     <t>contrasts</t>
@@ -12044,7 +12044,7 @@
     <t>02_HRvLR_groups/02_Protein_Contrasts/c_data/protein_contrasts.xlsx</t>
   </si>
   <si>
-    <t>f3294b7f02df2c8ee462be5604fcd0a5</t>
+    <t>e02599bb8f2c5a55f975346edd987fb0</t>
   </si>
   <si>
     <t>BiocGenerics</t>

</xml_diff>

<commit_message>
rerun the whole pipeline through the new run_all.R; results unchanged, 571 tests pass
</commit_message>
<xml_diff>
--- a/01_Processing/Figures/S01_QC/c_data/s01_qc.xlsx
+++ b/01_Processing/Figures/S01_QC/c_data/s01_qc.xlsx
@@ -12017,7 +12017,7 @@
     <t>01_Processing/01_Protein_Filtering/c_data/protein_filtering.xlsx</t>
   </si>
   <si>
-    <t>4854fa7ac6d2b74a44ea62851a66ea96</t>
+    <t>042ef917b7a47f9d5383779de262c03b</t>
   </si>
   <si>
     <t>normalize</t>
@@ -12026,7 +12026,7 @@
     <t>01_Processing/02_Normalisation/c_data/normalisation.xlsx</t>
   </si>
   <si>
-    <t>3f7dcfb017ee1077ac79f1a11c4cab5f</t>
+    <t>a4d88ef82050f32ecb819f1a7bae9bba</t>
   </si>
   <si>
     <t>quantify</t>
@@ -12035,7 +12035,7 @@
     <t>01_Processing/03_Quantification/c_data/quantification.xlsx</t>
   </si>
   <si>
-    <t>cdd28d73ea380e8e956c212adbcd2d74</t>
+    <t>e7097e9257459c7138e5e41e83efd467</t>
   </si>
   <si>
     <t>contrasts</t>
@@ -12044,7 +12044,7 @@
     <t>02_HRvLR_groups/02_Protein_Contrasts/c_data/protein_contrasts.xlsx</t>
   </si>
   <si>
-    <t>e02599bb8f2c5a55f975346edd987fb0</t>
+    <t>0d6cf853ff8d0d35c8767a6734aeecb9</t>
   </si>
   <si>
     <t>BiocGenerics</t>

</xml_diff>